<commit_message>
auto: D03·A02 — 로그인(UI-PAR-000/FN-PAR-00-01) 추가
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Audit/JJ_PD_IP_D03_메뉴구조도_v1.3_이노팸.xlsx
+++ b/Audit/JJ_PD_IP_D03_메뉴구조도_v1.3_이노팸.xlsx
@@ -4536,7 +4536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="11.83203125" bestFit="1" customWidth="1" style="11" min="1" max="2"/>
@@ -4638,12 +4638,12 @@
     <row r="5" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>UI-PAR-001</t>
+          <t>UI-PAR-000</t>
         </is>
       </c>
       <c r="B5" s="54" t="inlineStr">
         <is>
-          <t>대시보드</t>
+          <t>로그인</t>
         </is>
       </c>
       <c r="C5" s="55" t="n"/>
@@ -4656,12 +4656,12 @@
     <row r="6" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>UI-PAR-002</t>
+          <t>UI-PAR-001</t>
         </is>
       </c>
       <c r="B6" s="54" t="inlineStr">
         <is>
-          <t>민원현황</t>
+          <t>대시보드</t>
         </is>
       </c>
       <c r="C6" s="55" t="n"/>
@@ -4674,12 +4674,12 @@
     <row r="7" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>UI-PAR-003</t>
-        </is>
-      </c>
-      <c r="B7" s="56" t="inlineStr">
-        <is>
-          <t>분석∙시뮬레이션</t>
+          <t>UI-PAR-002</t>
+        </is>
+      </c>
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t>민원현황</t>
         </is>
       </c>
       <c r="C7" s="55" t="n"/>
@@ -4690,18 +4690,18 @@
       <c r="H7" s="39" t="n"/>
     </row>
     <row r="8" ht="15" customFormat="1" customHeight="1" s="10">
-      <c r="A8" s="20" t="n"/>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>UI-PAR-003-01</t>
-        </is>
-      </c>
-      <c r="D8" s="57" t="inlineStr">
-        <is>
-          <t>불법 주차 집중 구역 분석</t>
-        </is>
-      </c>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>UI-PAR-003</t>
+        </is>
+      </c>
+      <c r="B8" s="56" t="inlineStr">
+        <is>
+          <t>분석∙시뮬레이션</t>
+        </is>
+      </c>
+      <c r="C8" s="55" t="n"/>
+      <c r="D8" s="55" t="n"/>
       <c r="E8" s="55" t="n"/>
       <c r="F8" s="55" t="n"/>
       <c r="G8" s="55" t="n"/>
@@ -4712,12 +4712,12 @@
       <c r="B9" s="20" t="n"/>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-003-02</t>
+          <t>UI-PAR-003-01</t>
         </is>
       </c>
       <c r="D9" s="57" t="inlineStr">
         <is>
-          <t>정책 효과 시뮬레이션</t>
+          <t>불법 주차 집중 구역 분석</t>
         </is>
       </c>
       <c r="E9" s="55" t="n"/>
@@ -4730,31 +4730,30 @@
       <c r="B10" s="20" t="n"/>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-003-03</t>
+          <t>UI-PAR-003-02</t>
         </is>
       </c>
       <c r="D10" s="57" t="inlineStr">
         <is>
-          <t>생활권 시뮬레이션</t>
+          <t>정책 효과 시뮬레이션</t>
         </is>
       </c>
       <c r="E10" s="55" t="n"/>
       <c r="F10" s="55" t="n"/>
       <c r="G10" s="55" t="n"/>
       <c r="H10" s="39" t="n"/>
-      <c r="J10" s="13" t="n"/>
     </row>
     <row r="11" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="A11" s="20" t="n"/>
       <c r="B11" s="20" t="n"/>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-003-04</t>
+          <t>UI-PAR-003-03</t>
         </is>
       </c>
       <c r="D11" s="57" t="inlineStr">
         <is>
-          <t>구역추천</t>
+          <t>생활권 시뮬레이션</t>
         </is>
       </c>
       <c r="E11" s="55" t="n"/>
@@ -4768,12 +4767,12 @@
       <c r="B12" s="20" t="n"/>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-003-05</t>
+          <t>UI-PAR-003-04</t>
         </is>
       </c>
       <c r="D12" s="57" t="inlineStr">
         <is>
-          <t>투자우선순위 보드</t>
+          <t>구역추천</t>
         </is>
       </c>
       <c r="E12" s="55" t="n"/>
@@ -4783,36 +4782,37 @@
       <c r="J12" s="13" t="n"/>
     </row>
     <row r="13" ht="15" customFormat="1" customHeight="1" s="10">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>UI-PAR-004</t>
-        </is>
-      </c>
-      <c r="B13" s="56" t="inlineStr">
-        <is>
-          <t>보고서∙알림</t>
-        </is>
-      </c>
-      <c r="C13" s="55" t="n"/>
-      <c r="D13" s="55" t="n"/>
+      <c r="A13" s="20" t="n"/>
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>UI-PAR-003-05</t>
+        </is>
+      </c>
+      <c r="D13" s="57" t="inlineStr">
+        <is>
+          <t>투자우선순위 보드</t>
+        </is>
+      </c>
       <c r="E13" s="55" t="n"/>
       <c r="F13" s="55" t="n"/>
       <c r="G13" s="55" t="n"/>
       <c r="H13" s="39" t="n"/>
+      <c r="J13" s="13" t="n"/>
     </row>
     <row r="14" ht="15" customFormat="1" customHeight="1" s="10">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>UI-PAR-004-01</t>
-        </is>
-      </c>
-      <c r="D14" s="57" t="inlineStr">
-        <is>
-          <t>보고서 목록</t>
-        </is>
-      </c>
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>UI-PAR-004</t>
+        </is>
+      </c>
+      <c r="B14" s="56" t="inlineStr">
+        <is>
+          <t>보고서∙알림</t>
+        </is>
+      </c>
+      <c r="C14" s="55" t="n"/>
+      <c r="D14" s="55" t="n"/>
       <c r="E14" s="55" t="n"/>
       <c r="F14" s="55" t="n"/>
       <c r="G14" s="55" t="n"/>
@@ -4823,12 +4823,12 @@
       <c r="B15" s="20" t="n"/>
       <c r="C15" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-004-02</t>
+          <t>UI-PAR-004-01</t>
         </is>
       </c>
       <c r="D15" s="57" t="inlineStr">
         <is>
-          <t>보고서 관리</t>
+          <t>보고서 목록</t>
         </is>
       </c>
       <c r="E15" s="55" t="n"/>
@@ -4841,12 +4841,12 @@
       <c r="B16" s="20" t="n"/>
       <c r="C16" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-004-03</t>
+          <t>UI-PAR-004-02</t>
         </is>
       </c>
       <c r="D16" s="57" t="inlineStr">
         <is>
-          <t>위험단계 알림 조회</t>
+          <t>보고서 관리</t>
         </is>
       </c>
       <c r="E16" s="55" t="n"/>
@@ -4859,12 +4859,12 @@
       <c r="B17" s="20" t="n"/>
       <c r="C17" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-004-04</t>
+          <t>UI-PAR-004-03</t>
         </is>
       </c>
       <c r="D17" s="57" t="inlineStr">
         <is>
-          <t>위험단계 알림 관리</t>
+          <t>위험단계 알림 조회</t>
         </is>
       </c>
       <c r="E17" s="55" t="n"/>
@@ -4873,18 +4873,18 @@
       <c r="H17" s="39" t="n"/>
     </row>
     <row r="18" ht="15" customFormat="1" customHeight="1" s="10">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>UI-PAR-005</t>
-        </is>
-      </c>
-      <c r="B18" s="54" t="inlineStr">
-        <is>
-          <t>AI 어시스턴트</t>
-        </is>
-      </c>
-      <c r="C18" s="55" t="n"/>
-      <c r="D18" s="55" t="n"/>
+      <c r="A18" s="20" t="n"/>
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>UI-PAR-004-04</t>
+        </is>
+      </c>
+      <c r="D18" s="57" t="inlineStr">
+        <is>
+          <t>위험단계 알림 관리</t>
+        </is>
+      </c>
       <c r="E18" s="55" t="n"/>
       <c r="F18" s="55" t="n"/>
       <c r="G18" s="55" t="n"/>
@@ -4893,12 +4893,12 @@
     <row r="19" ht="15" customFormat="1" customHeight="1" s="10">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>UI-PAR-006</t>
+          <t>UI-PAR-005</t>
         </is>
       </c>
       <c r="B19" s="54" t="inlineStr">
         <is>
-          <t>설정</t>
+          <t>AI 어시스턴트</t>
         </is>
       </c>
       <c r="C19" s="55" t="n"/>
@@ -4909,18 +4909,18 @@
       <c r="H19" s="39" t="n"/>
     </row>
     <row r="20" ht="15" customFormat="1" customHeight="1" s="10">
-      <c r="A20" s="20" t="n"/>
-      <c r="B20" s="20" t="n"/>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>UI-PAR-006-01</t>
-        </is>
-      </c>
-      <c r="D20" s="57" t="inlineStr">
-        <is>
-          <t>메뉴 권한 관리</t>
-        </is>
-      </c>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>UI-PAR-006</t>
+        </is>
+      </c>
+      <c r="B20" s="54" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="C20" s="55" t="n"/>
+      <c r="D20" s="55" t="n"/>
       <c r="E20" s="55" t="n"/>
       <c r="F20" s="55" t="n"/>
       <c r="G20" s="55" t="n"/>
@@ -4931,18 +4931,36 @@
       <c r="B21" s="20" t="n"/>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>UI-PAR-006-02</t>
+          <t>UI-PAR-006-01</t>
         </is>
       </c>
       <c r="D21" s="57" t="inlineStr">
         <is>
-          <t>분석 지표 가중치 설정</t>
+          <t>메뉴 권한 관리</t>
         </is>
       </c>
       <c r="E21" s="55" t="n"/>
       <c r="F21" s="55" t="n"/>
       <c r="G21" s="55" t="n"/>
       <c r="H21" s="39" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="n"/>
+      <c r="B22" s="20" t="n"/>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>UI-PAR-006-02</t>
+        </is>
+      </c>
+      <c r="D22" s="57" t="inlineStr">
+        <is>
+          <t>분석 지표 가중치 설정</t>
+        </is>
+      </c>
+      <c r="E22" s="55" t="n"/>
+      <c r="F22" s="55" t="n"/>
+      <c r="G22" s="55" t="n"/>
+      <c r="H22" s="39" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">

</xml_diff>